<commit_message>
Updated PELCA Device Designer files: - IGBT manufacturing inventory - Python script for impact assessment - File requirements.txt - Impact assessment results - Instructions on how to use the PELCA Device Designer tools - Associated images and illustrations
</commit_message>
<xml_diff>
--- a/Input example/inputExample_v1.4.0_Efuse.xlsx
+++ b/Input example/inputExample_v1.4.0_Efuse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guillemet\Documents\PELCA_internal\Input example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27D094EF-A17A-4A19-9F18-6B5A31C08E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45CA00B3-33B6-4657-8B82-82240AC10054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PELCA - Legend | License" sheetId="21" r:id="rId1"/>
@@ -2723,10 +2723,10 @@
     </r>
   </si>
   <si>
-    <t>C:\Users\guillemet\Documents\PELCA_internal\Input example</t>
-  </si>
-  <si>
-    <t>/Users/guillemet/Downloads/ecoinvent 3.9.1_cutoff_ecoSpold02/datasets</t>
+    <t>/Users/username/Downloads/ecoinvent 3.9.1_cutoff_ecoSpold02/datasets</t>
+  </si>
+  <si>
+    <t>C:\Users\username\filepath</t>
   </si>
 </sst>
 </file>
@@ -54691,7 +54691,7 @@
         <v>31</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>32</v>
@@ -54742,7 +54742,7 @@
         <v>40</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
Minor updates of the PELCA Device Designer files (instructions.md).
</commit_message>
<xml_diff>
--- a/Input example/inputExample_v1.4.0_Efuse.xlsx
+++ b/Input example/inputExample_v1.4.0_Efuse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guillemet\Documents\PELCA_internal\Input example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45CA00B3-33B6-4657-8B82-82240AC10054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9DBB0D-BB5E-4E0D-88A0-645C50FA0483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PELCA - Legend | License" sheetId="21" r:id="rId1"/>
@@ -2417,13 +2417,6 @@
   </si>
   <si>
     <t>Electricity cost (€/kWh)</t>
-  </si>
-  <si>
-    <t>A RU (Reference Unit) can include multiple units. For example:
-- RU: 4 NP-type capacitors
-- Unit: 1 NP-type capacitor
-The exchange flows for each RU are defined based on a single unit.
-If the RU consists of N units, this is indicated in the 'scaling factor' column of the last row by 1/N. This cell shows that the flows defined for one unit (in the column 'quantity') represent 1/N of the flows for the total RU. Therefore, the flows for the RU correspond to N times the flows of a single unit.</t>
   </si>
   <si>
     <t>The tool allows models the diagnosis associated with the system, specifically detailing the replacement scenarios when a fault occurs. This includes identifying what components are replaced within the system, To achieve this, this sheet constructs the Replacement Matrix (RM). The numbers in the matrix represent the probability to replace each RU when a specific RU fails, with values ranging from 0 to 1. Row indices represent faults in a specific RU (e.g., Fault RU1), while column indices represent the RUs to be replaced (e.g., RU1). To clarify, consider an example with 2 RUs, resulting in a 2x2 matrix. In this example, if the value in the first row, first column (Fault RU1 ; RU1) is 1, and the value in the first row, second column (Fault RU1 ; RU2) is 0.6, this means that when a fault occurs in RU1, there is 100% probability of replacing RU1 and 60% probabilitu of replacing RU2 according to the diagnosis.</t>
@@ -2727,6 +2720,13 @@
   </si>
   <si>
     <t>C:\Users\username\filepath</t>
+  </si>
+  <si>
+    <t>A RU (Reference Unit) can include multiple units. For example:
+- RU: 4 NP-type capacitors
+- Unit: 1 NP-type capacitor
+The exchange flows for each RU are defined based on a single unit.
+If the RU consists of N units, this is indicated in the 'scaling factor' column of the last row by N. This cell shows that the flows defined for a single unit (in the column 'quantity') represent 1/N of the flows for the total RU. Therefore, the flows for the total RU correspond to N times the flows of a single unit. Example: the RU is a power switch embedding 4 power dice in parallel --&gt; the listed exchanges corresponds to the flows for the manufacturing of 1 power die ; the cell of column D ('scaling factor'), last row indicates 4 ; the cell of column E ('amount'), last row automatically indicates 1/N = 0,25 ; this means that the amounts of all the listed flows will be divided by 0,25 (i.e. multiplied by 4) when computing the manufacturing impacts of this RU.</t>
   </si>
 </sst>
 </file>
@@ -12798,22 +12798,22 @@
       <c r="E10" s="316"/>
       <c r="F10" s="316"/>
       <c r="G10" s="317" t="s">
+        <v>778</v>
+      </c>
+      <c r="H10" s="318" t="s">
         <v>779</v>
-      </c>
-      <c r="H10" s="318" t="s">
-        <v>780</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" thickBot="1">
       <c r="F11" s="324" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="G11" s="325"/>
       <c r="H11" s="325"/>
     </row>
     <row r="12" spans="1:8">
       <c r="B12" s="326" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C12" s="327"/>
       <c r="D12" s="327"/>
@@ -12829,7 +12829,7 @@
     <row r="14" spans="1:8">
       <c r="B14" s="319"/>
       <c r="C14" s="320" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="H14" s="197"/>
     </row>
@@ -12840,7 +12840,7 @@
     <row r="16" spans="1:8">
       <c r="B16" s="321"/>
       <c r="C16" s="320" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="H16" s="197"/>
     </row>
@@ -12850,10 +12850,10 @@
     </row>
     <row r="18" spans="2:8" ht="15" thickBot="1">
       <c r="B18" s="322" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="C18" s="323" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="D18" s="307"/>
       <c r="E18" s="307"/>
@@ -12864,7 +12864,7 @@
     <row r="19" spans="2:8" ht="15" thickBot="1"/>
     <row r="20" spans="2:8" ht="15" customHeight="1">
       <c r="B20" s="329" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C20" s="330"/>
       <c r="D20" s="330"/>
@@ -14401,7 +14401,7 @@
     <col min="2" max="2" width="5.6640625" style="63" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="63" customWidth="1"/>
     <col min="4" max="4" width="19.6640625" style="63" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.33203125" style="63" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49" style="63" customWidth="1"/>
     <col min="6" max="6" width="12.33203125" style="63" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.33203125" style="63" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="63" bestFit="1" customWidth="1"/>
@@ -42241,7 +42241,7 @@
   <dimension ref="A1:J416"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="48.109375" style="33" customWidth="1"/>
+    <col min="1" max="1" width="74.44140625" style="33" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.33203125" style="33" customWidth="1"/>
     <col min="3" max="3" width="12.44140625" style="33" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.77734375" style="33" bestFit="1" customWidth="1"/>
@@ -42253,12 +42253,12 @@
     <col min="10" max="16384" width="10.6640625" style="33"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="111" customHeight="1">
+    <row r="1" spans="1:10" ht="148.80000000000001" customHeight="1">
       <c r="A1" s="22" t="s">
         <v>30</v>
       </c>
       <c r="B1" s="338" t="s">
-        <v>777</v>
+        <v>789</v>
       </c>
       <c r="C1" s="338"/>
       <c r="D1" s="338"/>
@@ -48290,11 +48290,11 @@
         <v>9</v>
       </c>
       <c r="D194" s="211">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E194" s="252">
         <f>B194/D194</f>
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F194" s="251" t="str">
         <f>$B$2</f>
@@ -54691,7 +54691,7 @@
         <v>31</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>32</v>
@@ -54742,7 +54742,7 @@
         <v>40</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>41</v>
@@ -55141,7 +55141,7 @@
         <v>30</v>
       </c>
       <c r="B2" s="341" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C2" s="342"/>
       <c r="D2" s="342"/>

</xml_diff>